<commit_message>
DB 파일 업데이트: ReelCarePam.xlsx 변경
</commit_message>
<xml_diff>
--- a/DB/ReelCarePam.xlsx
+++ b/DB/ReelCarePam.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="814" uniqueCount="560">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="922" uniqueCount="661">
   <si>
     <t>위탁날짜</t>
   </si>
@@ -1706,11 +1706,312 @@
   </si>
   <si>
     <t>판매포인트</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>판매포인트</t>
-    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>이그지스트는 다이와 스피닝릴의 정점에 있는 모델이라, 중고로 나와도 반기시는 분들이 많습니다. 연식이 있어도 관리만 잘 되어 있으면 여전히 문의가 꾸준한 편이고요. 릴케어팜에서 꼼꼼히 검수하고 손봐서 내보내면 구매자분들도 더 안심하고 선택하십니다.</t>
+  </si>
+  <si>
+    <t>에어리티는 브랜드를 대표하는 플래그십답게, 매물이 나오면 마니아들의 관심이 먼저 쏠리는 릴입니다. 위탁 주시면 검수와 오버홀을 거쳐 상태 그대로 정직하게 소개해 드리겠습니다.</t>
+  </si>
+  <si>
+    <t>에어리티는 크게 튀는 스펙은 아니지만 그만큼 실속 있다는 인식이 있어 수요가 꾸준합니다. 배스 하시는 분들한테 물어보면 이름을 다 알 정도입니다. 릴케어팜에서 꼼꼼히 검수하고 손봐서 내보내면 구매자분들도 더 안심하고 선택하십니다.</t>
+  </si>
+  <si>
+    <t>세르테이트는 가격과 성능의 밸런스가 좋아서 꾸준히 찾는 분들이 있는 스테디셀러입니다. 특정 장르에 국한되지 않고 여러 상황에서 무난히 쓸 수 있습니다. 검수 후 상태를 투명하게 공개해서 내보내면, 구매하시는 분들도 믿고 결정하시더라고요.</t>
+  </si>
+  <si>
+    <t>세르테이트를 두루 무난하게 쓸 수 있다는 평이 많아, 중고 거래도 활발한 편에 속합니다. 쇼어지깅·인쇼어 위주로 쓰시는 분들이 많이 찾는 편입니다. 릴케어팜을 통해 위탁하시면 전문 검수와 정비를 거쳐 훨씬 수월하게 판매하실 수 있습니다.</t>
+  </si>
+  <si>
+    <t>루비아스는 성능 대비 평가가 좋은 편이라, 상태만 괜찮으면 금방 새 주인을 만납니다. 특정 장르에 국한되지 않고 여러 상황에서 무난히 쓸 수 있습니다. 릴케어팜을 통해 위탁하시면 전문 검수와 정비를 거쳐 훨씬 수월하게 판매하실 수 있습니다.</t>
+  </si>
+  <si>
+    <t>루비아스를 두루 무난하게 쓸 수 있다는 평이 많아, 중고 거래도 활발한 편에 속합니다. 장르를 가리지 않고 두루 쓰인다는 점도 강점입니다. 저희 쪽에서 오버홀까지 마치고 판매하면 신뢰도가 올라가서 거래가 한결 수월해집니다.</t>
+  </si>
+  <si>
+    <t>발리스틱은 가격과 성능의 밸런스가 좋아서 꾸준히 찾는 분들이 있는 스테디셀러입니다. 특정 장르에 국한되지 않고 여러 상황에서 무난히 쓸 수 있습니다. 저희 쪽에서 오버홀까지 마치고 판매하면 신뢰도가 올라가서 거래가 한결 수월해집니다.</t>
+  </si>
+  <si>
+    <t>칼디아를 처음 시작하는 분들이 많이 선택하다 보니, 중고 물량도 꾸준히 순환됩니다. 특정 장르에 국한되지 않고 여러 상황에서 무난히 쓸 수 있습니다. 검수 후 상태를 투명하게 공개해서 내보내면, 구매하시는 분들도 믿고 결정하시더라고요.</t>
+  </si>
+  <si>
+    <t>렉사는 가격과 성능의 밸런스가 좋아서 꾸준히 찾는 분들이 있는 스테디셀러입니다. 선상 지깅 즐기는 분들에게 특히 반응이 좋은 편입니다. 검수 후 상태를 투명하게 공개해서 내보내면, 구매하시는 분들도 믿고 결정하시더라고요.</t>
+  </si>
+  <si>
+    <t>프림스는 가성비 좋은 입문작으로 알려져 있어서, 상태 좋은 매물은 크게 오래 기다리지 않고 나갑니다. 검수 후 상태를 투명하게 공개해서 내보내면, 구매하시는 분들도 믿고 결정하시더라고요.</t>
+  </si>
+  <si>
+    <t>레갈리스는 부담 없는 가격대라 입문자들이 많이 찾는 만큼, 중고로도 회전이 빠른 편입니다. 릴케어팜을 통해 위탁하시면 전문 검수와 정비를 거쳐 훨씬 수월하게 판매하실 수 있습니다.</t>
+  </si>
+  <si>
+    <t>레브로스를 처음 시작하는 분들이 많이 선택하다 보니, 중고 물량도 꾸준히 순환됩니다. 릴케어팜을 통해 위탁하시면 전문 검수와 정비를 거쳐 훨씬 수월하게 판매하실 수 있습니다.</t>
+  </si>
+  <si>
+    <t>스텔라는 스피닝릴 중에서도 최고봉으로 꼽히는 만큼, 매물이 나오면 마니아분들이 먼저 알아보고 연락 주시는 릴입니다. 상태만 잘 관리되어 있으면 오래 기다리지 않고 거래가 성사되는 편이고요. 위탁 주시면 검수와 오버홀을 거쳐 상태 그대로 정직하게 소개해 드리겠습니다.</t>
+  </si>
+  <si>
+    <t>뱅퀴시를 두루 무난하게 쓸 수 있다는 평이 많아, 중고 거래도 활발한 편에 속합니다. 특정 장르에 국한되지 않고 여러 상황에서 무난히 쓸 수 있습니다. 맡겨주시면 상태 점검부터 오버홀까지 해서, 제값 받고 팔릴 수 있게 도와드리겠습니다.</t>
+  </si>
+  <si>
+    <t>트윈파워는 가격과 성능의 밸런스가 좋아서 꾸준히 찾는 분들이 있는 스테디셀러입니다. 위탁 주시면 검수와 오버홀을 거쳐 상태 그대로 정직하게 소개해 드리겠습니다.</t>
+  </si>
+  <si>
+    <t>스트라딕을 두루 무난하게 쓸 수 있다는 평이 많아, 중고 거래도 활발한 편에 속합니다. 특정 장르에 국한되지 않고 여러 상황에서 무난히 쓸 수 있습니다. 맡겨주시면 상태 점검부터 오버홀까지 해서, 제값 받고 팔릴 수 있게 도와드리겠습니다.</t>
+  </si>
+  <si>
+    <t>울테그라를 처음 시작하는 분들이 많이 선택하다 보니, 중고 물량도 꾸준히 순환됩니다. 장르를 가리지 않고 두루 쓰인다는 점도 강점입니다. 위탁 주시면 검수와 오버홀을 거쳐 상태 그대로 정직하게 소개해 드리겠습니다.</t>
+  </si>
+  <si>
+    <t>사하라는 부담 없는 가격대라 입문자들이 많이 찾는 만큼, 중고로도 회전이 빠른 편입니다. 맡겨주시면 상태 점검부터 오버홀까지 해서, 제값 받고 팔릴 수 있게 도와드리겠습니다.</t>
+  </si>
+  <si>
+    <t>세도나는 부담 없는 가격대라 입문자들이 많이 찾는 만큼, 중고로도 회전이 빠른 편입니다. 검수 후 상태를 투명하게 공개해서 내보내면, 구매하시는 분들도 믿고 결정하시더라고요.</t>
+  </si>
+  <si>
+    <t>시에나는 부담 없는 가격대라 입문자들이 많이 찾는 만큼, 중고로도 회전이 빠른 편입니다. 원투 위주로 쓰시는 분들이 많이 찾는 편입니다. 릴케어팜에서 꼼꼼히 검수하고 손봐서 내보내면 구매자분들도 더 안심하고 선택하십니다.</t>
+  </si>
+  <si>
+    <t>워낙 인지도가 높은 볼란테를 찾는 분들이 꾸준해서, 컨디션만 받쳐주면 거래는 어렵지 않게 성사됩니다. 검수 후 상태를 투명하게 공개해서 내보내면, 구매하시는 분들도 믿고 결정하시더라고요.</t>
+  </si>
+  <si>
+    <t>하데스 프로는 크게 튀는 스펙은 아니지만 그만큼 실속 있다는 인식이 있어 수요가 꾸준합니다. 장르를 가리지 않고 두루 쓰인다는 점도 강점입니다. 맡겨주시면 상태 점검부터 오버홀까지 해서, 제값 받고 팔릴 수 있게 도와드리겠습니다.</t>
+  </si>
+  <si>
+    <t>하데스는 부담 없는 가격대라 입문자들이 많이 찾는 만큼, 중고로도 회전이 빠른 편입니다. 배스 즐기는 분들에게 특히 반응이 좋은 편입니다. 맡겨주시면 상태 점검부터 오버홀까지 해서, 제값 받고 팔릴 수 있게 도와드리겠습니다.</t>
+  </si>
+  <si>
+    <t>코티나는 부담 없는 가격대라 입문자들이 많이 찾는 만큼, 중고로도 회전이 빠른 편입니다. 쇼어지깅·인쇼어 위주로 쓰시는 분들이 많이 찾는 편입니다. 저희 쪽에서 오버홀까지 마치고 판매하면 신뢰도가 올라가서 거래가 한결 수월해집니다.</t>
+  </si>
+  <si>
+    <t>토리노 서프는 크게 튀는 스펙은 아니지만 그만큼 실속 있다는 인식이 있어 수요가 꾸준합니다. 원투 위주로 쓰시는 분들이 많이 찾는 편입니다. 저희 쪽에서 오버홀까지 마치고 판매하면 신뢰도가 올라가서 거래가 한결 수월해집니다.</t>
+  </si>
+  <si>
+    <t>커맨더 프로는 가성비 좋은 입문작으로 알려져 있어서, 상태 좋은 매물은 크게 오래 기다리지 않고 나갑니다. 특정 장르에 국한되지 않고 여러 상황에서 무난히 쓸 수 있습니다. 릴케어팜에서 꼼꼼히 검수하고 손봐서 내보내면 구매자분들도 더 안심하고 선택하십니다.</t>
+  </si>
+  <si>
+    <t>넥스텀은 부담 없는 가격대라 입문자들이 많이 찾는 만큼, 중고로도 회전이 빠른 편입니다. 특정 장르에 국한되지 않고 여러 상황에서 무난히 쓸 수 있습니다. 저희 쪽에서 오버홀까지 마치고 판매하면 신뢰도가 올라가서 거래가 한결 수월해집니다.</t>
+  </si>
+  <si>
+    <t>제논 스피닝은 브랜드를 대표하는 플래그십답게, 매물이 나오면 마니아들의 관심이 먼저 쏠리는 릴입니다. 장르를 가리지 않고 두루 쓰인다는 점도 강점입니다. 릴케어팜에서 꼼꼼히 검수하고 손봐서 내보내면 구매자분들도 더 안심하고 선택하십니다.</t>
+  </si>
+  <si>
+    <t>레보 MGX는 성능 대비 평가가 좋은 편이라, 상태만 괜찮으면 금방 새 주인을 만납니다. 맡겨주시면 상태 점검부터 오버홀까지 해서, 제값 받고 팔릴 수 있게 도와드리겠습니다.</t>
+  </si>
+  <si>
+    <t>레보 ALX 세타는 크게 튀는 스펙은 아니지만 그만큼 실속 있다는 인식이 있어 수요가 꾸준합니다. 특정 장르에 국한되지 않고 여러 상황에서 무난히 쓸 수 있습니다. 릴케어팜에서 꼼꼼히 검수하고 손봐서 내보내면 구매자분들도 더 안심하고 선택하십니다.</t>
+  </si>
+  <si>
+    <t>로간은 가격과 성능의 밸런스가 좋아서 꾸준히 찾는 분들이 있는 스테디셀러입니다. 특히 쇼어지깅·인쇼어 하시는 분들 사이에서 선호도가 높습니다. 릴케어팜을 통해 위탁하시면 전문 검수와 정비를 거쳐 훨씬 수월하게 판매하실 수 있습니다.</t>
+  </si>
+  <si>
+    <t>록사니 스피닝은 성능 대비 평가가 좋은 편이라, 상태만 괜찮으면 금방 새 주인을 만납니다. 장르를 가리지 않고 두루 쓰인다는 점도 강점입니다. 저희 쪽에서 오버홀까지 마치고 판매하면 신뢰도가 올라가서 거래가 한결 수월해집니다.</t>
+  </si>
+  <si>
+    <t>슈페리어를 두루 무난하게 쓸 수 있다는 평이 많아, 중고 거래도 활발한 편에 속합니다. 특정 장르에 국한되지 않고 여러 상황에서 무난히 쓸 수 있습니다. 릴케어팜에서 꼼꼼히 검수하고 손봐서 내보내면 구매자분들도 더 안심하고 선택하십니다.</t>
+  </si>
+  <si>
+    <t>카디날 3는 부담 없는 가격대라 입문자들이 많이 찾는 만큼, 중고로도 회전이 빠른 편입니다. 저희 쪽에서 오버홀까지 마치고 판매하면 신뢰도가 올라가서 거래가 한결 수월해집니다.</t>
+  </si>
+  <si>
+    <t>프라임 서프를 두루 무난하게 쓸 수 있다는 평이 많아, 중고 거래도 활발한 편에 속합니다. 릴케어팜에서 꼼꼼히 검수하고 손봐서 내보내면 구매자분들도 더 안심하고 선택하십니다.</t>
+  </si>
+  <si>
+    <t>코바4는 도요피싱을 대표하는 베이트릴로, 합리적인 가격과 성능 덕분에 꾸준히 인기가 있는 모델입니다. 배스낚시 입문자부터 중급자까지 폭넓게 사용하시고요. 중고시장에서도 거래가 안정적으로 이루어지는 편입니다. 맡겨주시면 상태 점검부터 오버홀까지 해서, 제값 받고 팔릴 수 있게 도와드리겠습니다.</t>
+  </si>
+  <si>
+    <t>코바 엘리트를 두루 무난하게 쓸 수 있다는 평이 많아, 중고 거래도 활발한 편에 속합니다. 피네스·계류 쪽 사용자층에서 유독 인지도가 높은 편이고요. 맡겨주시면 상태 점검부터 오버홀까지 해서, 제값 받고 팔릴 수 있게 도와드리겠습니다.</t>
+  </si>
+  <si>
+    <t>코바3는 소장 가치가 높은 상위 라인이라, 상태 좋은 개체는 오래 묵히지 않고 팔려나가는 편입니다. 특정 장르에 국한되지 않고 여러 상황에서 무난히 쓸 수 있습니다. 저희 쪽에서 오버홀까지 마치고 판매하면 신뢰도가 올라가서 거래가 한결 수월해집니다.</t>
+  </si>
+  <si>
+    <t>코바 라이트를 한 번 써본 분들의 만족도가 높다 보니, 재판매 수요도 꾸준한 편입니다. 검수 후 상태를 투명하게 공개해서 내보내면, 구매하시는 분들도 믿고 결정하시더라고요.</t>
+  </si>
+  <si>
+    <t>라이거30는 크게 튀는 스펙은 아니지만 그만큼 실속 있다는 인식이 있어 수요가 꾸준합니다. 배스 쪽 사용자층에서 유독 인지도가 높은 편이고요. 저희 쪽에서 오버홀까지 마치고 판매하면 신뢰도가 올라가서 거래가 한결 수월해집니다.</t>
+  </si>
+  <si>
+    <t>라이거30 DLC를 두루 무난하게 쓸 수 있다는 평이 많아, 중고 거래도 활발한 편에 속합니다. 릴케어팜을 통해 위탁하시면 전문 검수와 정비를 거쳐 훨씬 수월하게 판매하실 수 있습니다.</t>
+  </si>
+  <si>
+    <t>올터레인 DLC는 크게 튀는 스펙은 아니지만 그만큼 실속 있다는 인식이 있어 수요가 꾸준합니다. 특정 장르에 국한되지 않고 여러 상황에서 무난히 쓸 수 있습니다. 저희 쪽에서 오버홀까지 마치고 판매하면 신뢰도가 올라가서 거래가 한결 수월해집니다.</t>
+  </si>
+  <si>
+    <t>올터레인 BG는 가격과 성능의 밸런스가 좋아서 꾸준히 찾는 분들이 있는 스테디셀러입니다. 참돔 타이라바 하시는 분들한테 물어보면 이름을 다 알 정도입니다. 맡겨주시면 상태 점검부터 오버홀까지 해서, 제값 받고 팔릴 수 있게 도와드리겠습니다.</t>
+  </si>
+  <si>
+    <t>라이거30 SW는 가격과 성능의 밸런스가 좋아서 꾸준히 찾는 분들이 있는 스테디셀러입니다. 장르를 가리지 않고 두루 쓰인다는 점도 강점입니다. 릴케어팜을 통해 위탁하시면 전문 검수와 정비를 거쳐 훨씬 수월하게 판매하실 수 있습니다.</t>
+  </si>
+  <si>
+    <t>올터레인4를 두루 무난하게 쓸 수 있다는 평이 많아, 중고 거래도 활발한 편에 속합니다. 배스 쪽 사용자층에서 유독 인지도가 높은 편이고요. 저희 쪽에서 오버홀까지 마치고 판매하면 신뢰도가 올라가서 거래가 한결 수월해집니다.</t>
+  </si>
+  <si>
+    <t>루비나 블랙 스페셜을 두루 무난하게 쓸 수 있다는 평이 많아, 중고 거래도 활발한 편에 속합니다. 특정 장르에 국한되지 않고 여러 상황에서 무난히 쓸 수 있습니다. 릴케어팜을 통해 위탁하시면 전문 검수와 정비를 거쳐 훨씬 수월하게 판매하실 수 있습니다.</t>
+  </si>
+  <si>
+    <t>헤비 듀티를 두루 무난하게 쓸 수 있다는 평이 많아, 중고 거래도 활발한 편에 속합니다. 맡겨주시면 상태 점검부터 오버홀까지 해서, 제값 받고 팔릴 수 있게 도와드리겠습니다.</t>
+  </si>
+  <si>
+    <t>루비나를 한 번 써본 분들의 만족도가 높다 보니, 재판매 수요도 꾸준한 편입니다. 장르를 가리지 않고 두루 쓰인다는 점도 강점입니다. 검수 후 상태를 투명하게 공개해서 내보내면, 구매하시는 분들도 믿고 결정하시더라고요.</t>
+  </si>
+  <si>
+    <t>우라노 인쇼어는 부담 없는 가격대라 입문자들이 많이 찾는 만큼, 중고로도 회전이 빠른 편입니다. 장르를 가리지 않고 두루 쓰인다는 점도 강점입니다. 맡겨주시면 상태 점검부터 오버홀까지 해서, 제값 받고 팔릴 수 있게 도와드리겠습니다.</t>
+  </si>
+  <si>
+    <t>라그나 BG 라이트를 처음 시작하는 분들이 많이 선택하다 보니, 중고 물량도 꾸준히 순환됩니다. 위탁 주시면 검수와 오버홀을 거쳐 상태 그대로 정직하게 소개해 드리겠습니다.</t>
+  </si>
+  <si>
+    <t>우라노를 처음 시작하는 분들이 많이 선택하다 보니, 중고 물량도 꾸준히 순환됩니다. 장르를 가리지 않고 두루 쓰인다는 점도 강점입니다. 위탁 주시면 검수와 오버홀을 거쳐 상태 그대로 정직하게 소개해 드리겠습니다.</t>
+  </si>
+  <si>
+    <t>스쿠텀 레드는 부담 없는 가격대라 입문자들이 많이 찾는 만큼, 중고로도 회전이 빠른 편입니다. 특정 장르에 국한되지 않고 여러 상황에서 무난히 쓸 수 있습니다. 릴케어팜을 통해 위탁하시면 전문 검수와 정비를 거쳐 훨씬 수월하게 판매하실 수 있습니다.</t>
+  </si>
+  <si>
+    <t>라그나를 처음 시작하는 분들이 많이 선택하다 보니, 중고 물량도 꾸준히 순환됩니다. 저희 쪽에서 오버홀까지 마치고 판매하면 신뢰도가 올라가서 거래가 한결 수월해집니다.</t>
+  </si>
+  <si>
+    <t>리카온은 가성비 좋은 입문작으로 알려져 있어서, 상태 좋은 매물은 크게 오래 기다리지 않고 나갑니다. 장르를 가리지 않고 두루 쓰인다는 점도 강점입니다. 위탁 주시면 검수와 오버홀을 거쳐 상태 그대로 정직하게 소개해 드리겠습니다.</t>
+  </si>
+  <si>
+    <t>스티즈는 소장 가치가 높은 상위 라인이라, 상태 좋은 개체는 오래 묵히지 않고 팔려나가는 편입니다. 위탁 주시면 검수와 오버홀을 거쳐 상태 그대로 정직하게 소개해 드리겠습니다.</t>
+  </si>
+  <si>
+    <t>워낙 인지도가 높은 스티즈를 찾는 분들이 꾸준해서, 컨디션만 받쳐주면 거래는 어렵지 않게 성사됩니다. 검수 후 상태를 투명하게 공개해서 내보내면, 구매하시는 분들도 믿고 결정하시더라고요.</t>
+  </si>
+  <si>
+    <t>아드미라는 가격과 성능의 밸런스가 좋아서 꾸준히 찾는 분들이 있는 스테디셀러입니다. 릴케어팜을 통해 위탁하시면 전문 검수와 정비를 거쳐 훨씬 수월하게 판매하실 수 있습니다.</t>
+  </si>
+  <si>
+    <t>코우가는 가격과 성능의 밸런스가 좋아서 꾸준히 찾는 분들이 있는 스테디셀러입니다. 참돔 타이라바 하시는 분들한테 물어보면 이름을 다 알 정도입니다. 릴케어팜을 통해 위탁하시면 전문 검수와 정비를 거쳐 훨씬 수월하게 판매하실 수 있습니다.</t>
+  </si>
+  <si>
+    <t>질리언 SV TW는 여러 루어를 두루 운용할 수 있는 범용 베이트릴이라 꾸준히 찾는 분들이 있습니다. 내구성과 캐스팅 성능이 좋다는 평이 많아 배스낚시 하시는 분들 선호도가 높은 편이고요. 관리 상태가 좋으면 중고시장에서도 평가가 좋습니다. 릴케어팜을 통해 위탁하시면 전문 검수와 정비를 거쳐 훨씬 수월하게 판매하실 수 있습니다.</t>
+  </si>
+  <si>
+    <t>솔티스트 TW는 크게 튀는 스펙은 아니지만 그만큼 실속 있다는 인식이 있어 수요가 꾸준합니다. 에깅 위주로 쓰시는 분들이 많이 찾는 편입니다. 릴케어팜을 통해 위탁하시면 전문 검수와 정비를 거쳐 훨씬 수월하게 판매하실 수 있습니다.</t>
+  </si>
+  <si>
+    <t>알파스는 크게 튀는 스펙은 아니지만 그만큼 실속 있다는 인식이 있어 수요가 꾸준합니다. 맡겨주시면 상태 점검부터 오버홀까지 해서, 제값 받고 팔릴 수 있게 도와드리겠습니다.</t>
+  </si>
+  <si>
+    <t>알파스를 한 번 써본 분들의 만족도가 높다 보니, 재판매 수요도 꾸준한 편입니다. 장르를 가리지 않고 두루 쓰인다는 점도 강점입니다. 릴케어팜에서 꼼꼼히 검수하고 손봐서 내보내면 구매자분들도 더 안심하고 선택하십니다.</t>
+  </si>
+  <si>
+    <t>알파스는 상급기답게 완성도가 좋아서, 중고시장에서도 문의가 끊이지 않는 모델입니다. 맡겨주시면 상태 점검부터 오버홀까지 해서, 제값 받고 팔릴 수 있게 도와드리겠습니다.</t>
+  </si>
+  <si>
+    <t>타튤라는 크게 튀는 스펙은 아니지만 그만큼 실속 있다는 인식이 있어 수요가 꾸준합니다. 릴케어팜에서 꼼꼼히 검수하고 손봐서 내보내면 구매자분들도 더 안심하고 선택하십니다.</t>
+  </si>
+  <si>
+    <t>타튤라는 가격과 성능의 밸런스가 좋아서 꾸준히 찾는 분들이 있는 스테디셀러입니다. 장르를 가리지 않고 두루 쓰인다는 점도 강점입니다. 위탁 주시면 검수와 오버홀을 거쳐 상태 그대로 정직하게 소개해 드리겠습니다.</t>
+  </si>
+  <si>
+    <t>라이트게임은 크게 튀는 스펙은 아니지만 그만큼 실속 있다는 인식이 있어 수요가 꾸준합니다. 주꾸미·갑오징어 선상 즐기는 분들에게 특히 반응이 좋은 편입니다. 위탁 주시면 검수와 오버홀을 거쳐 상태 그대로 정직하게 소개해 드리겠습니다.</t>
+  </si>
+  <si>
+    <t>라이즈를 처음 시작하는 분들이 많이 선택하다 보니, 중고 물량도 꾸준히 순환됩니다. 장르를 가리지 않고 두루 쓰인다는 점도 강점입니다. 릴케어팜을 통해 위탁하시면 전문 검수와 정비를 거쳐 훨씬 수월하게 판매하실 수 있습니다.</t>
+  </si>
+  <si>
+    <t>라이트게임은 크게 튀는 스펙은 아니지만 그만큼 실속 있다는 인식이 있어 수요가 꾸준합니다. 특정 장르에 국한되지 않고 여러 상황에서 무난히 쓸 수 있습니다. 릴케어팜을 통해 위탁하시면 전문 검수와 정비를 거쳐 훨씬 수월하게 판매하실 수 있습니다.</t>
+  </si>
+  <si>
+    <t>프리드는 부담 없는 가격대라 입문자들이 많이 찾는 만큼, 중고로도 회전이 빠른 편입니다. 장르를 가리지 않고 두루 쓰인다는 점도 강점입니다. 맡겨주시면 상태 점검부터 오버홀까지 해서, 제값 받고 팔릴 수 있게 도와드리겠습니다.</t>
+  </si>
+  <si>
+    <t>PR 100는 가성비 좋은 입문작으로 알려져 있어서, 상태 좋은 매물은 크게 오래 기다리지 않고 나갑니다. 특정 장르에 국한되지 않고 여러 상황에서 무난히 쓸 수 있습니다. 위탁 주시면 검수와 오버홀을 거쳐 상태 그대로 정직하게 소개해 드리겠습니다.</t>
+  </si>
+  <si>
+    <t>안타레스는 배스 루어 낚시를 하는 분들 사이에서 손꼽히는 플래그십 베이트릴입니다. DC 브레이크 성능이 좋다는 인식이 있어서, 상태 좋은 매물은 오래 묵히지 않고 팔려나가는 편이고요. 위탁 주시면 검수와 오버홀을 거쳐 상태 그대로 정직하게 소개해 드리겠습니다.</t>
+  </si>
+  <si>
+    <t>캘커타 콘퀘스트는 크게 튀는 스펙은 아니지만 그만큼 실속 있다는 인식이 있어 수요가 꾸준합니다. 특정 장르에 국한되지 않고 여러 상황에서 무난히 쓸 수 있습니다. 위탁 주시면 검수와 오버홀을 거쳐 상태 그대로 정직하게 소개해 드리겠습니다.</t>
+  </si>
+  <si>
+    <t>캘커타 콘퀘스트를 두루 무난하게 쓸 수 있다는 평이 많아, 중고 거래도 활발한 편에 속합니다. 릴케어팜에서 꼼꼼히 검수하고 손봐서 내보내면 구매자분들도 더 안심하고 선택하십니다.</t>
+  </si>
+  <si>
+    <t>메타늄은 배스낚시 하시는 분들 사이에서 꾸준히 이름이 나오는 대표적인 베이트릴입니다. 무게가 가볍고 성능이 안정적이라 입문자부터 상급자까지 두루 선호하는 편이고요. 상태 좋은 물건은 중고로 나와도 비교적 빠르게 팔립니다. 위탁 주시면 검수와 오버홀을 거쳐 상태 그대로 정직하게 소개해 드리겠습니다.</t>
+  </si>
+  <si>
+    <t>알데바란은 이 라인업의 최상위 모델인 만큼, 중고로 나와도 반기는 분들이 많은 편입니다. 피네스·계류 쪽 사용자층에서 유독 인지도가 높은 편이고요. 위탁 주시면 검수와 오버홀을 거쳐 상태 그대로 정직하게 소개해 드리겠습니다.</t>
+  </si>
+  <si>
+    <t>엔게츠 프리미엄을 두루 무난하게 쓸 수 있다는 평이 많아, 중고 거래도 활발한 편에 속합니다. 특정 장르에 국한되지 않고 여러 상황에서 무난히 쓸 수 있습니다. 맡겨주시면 상태 점검부터 오버홀까지 해서, 제값 받고 팔릴 수 있게 도와드리겠습니다.</t>
+  </si>
+  <si>
+    <t>스콜피온은 크게 튀는 스펙은 아니지만 그만큼 실속 있다는 인식이 있어 수요가 꾸준합니다. 특정 장르에 국한되지 않고 여러 상황에서 무난히 쓸 수 있습니다. 검수 후 상태를 투명하게 공개해서 내보내면, 구매하시는 분들도 믿고 결정하시더라고요.</t>
+  </si>
+  <si>
+    <t>SLX는 부담 없는 가격대라 입문자들이 많이 찾는 만큼, 중고로도 회전이 빠른 편입니다. 장르를 가리지 않고 두루 쓰인다는 점도 강점입니다. 저희 쪽에서 오버홀까지 마치고 판매하면 신뢰도가 올라가서 거래가 한결 수월해집니다.</t>
+  </si>
+  <si>
+    <t>염월 BB를 처음 시작하는 분들이 많이 선택하다 보니, 중고 물량도 꾸준히 순환됩니다. 참돔 타이라바 즐기는 분들에게 특히 반응이 좋은 편입니다. 검수 후 상태를 투명하게 공개해서 내보내면, 구매하시는 분들도 믿고 결정하시더라고요.</t>
+  </si>
+  <si>
+    <t>바스원 XT는 가성비 좋은 입문작으로 알려져 있어서, 상태 좋은 매물은 크게 오래 기다리지 않고 나갑니다. 장르를 가리지 않고 두루 쓰인다는 점도 강점입니다. 저희 쪽에서 오버홀까지 마치고 판매하면 신뢰도가 올라가서 거래가 한결 수월해집니다.</t>
+  </si>
+  <si>
+    <t>아이오닉스 인쇼어는 가격과 성능의 밸런스가 좋아서 꾸준히 찾는 분들이 있는 스테디셀러입니다. 장르를 가리지 않고 두루 쓰인다는 점도 강점입니다. 릴케어팜에서 꼼꼼히 검수하고 손봐서 내보내면 구매자분들도 더 안심하고 선택하십니다.</t>
+  </si>
+  <si>
+    <t>아폴로 티탄 SW는 성능 대비 평가가 좋은 편이라, 상태만 괜찮으면 금방 새 주인을 만납니다. 특정 장르에 국한되지 않고 여러 상황에서 무난히 쓸 수 있습니다. 릴케어팜을 통해 위탁하시면 전문 검수와 정비를 거쳐 훨씬 수월하게 판매하실 수 있습니다.</t>
+  </si>
+  <si>
+    <t>아폴로 SW를 두루 무난하게 쓸 수 있다는 평이 많아, 중고 거래도 활발한 편에 속합니다. 장르를 가리지 않고 두루 쓰인다는 점도 강점입니다. 릴케어팜을 통해 위탁하시면 전문 검수와 정비를 거쳐 훨씬 수월하게 판매하실 수 있습니다.</t>
+  </si>
+  <si>
+    <t>알파드 LITE를 처음 시작하는 분들이 많이 선택하다 보니, 중고 물량도 꾸준히 순환됩니다. 릴케어팜에서 꼼꼼히 검수하고 손봐서 내보내면 구매자분들도 더 안심하고 선택하십니다.</t>
+  </si>
+  <si>
+    <t>G 타코 4는 크게 튀는 스펙은 아니지만 그만큼 실속 있다는 인식이 있어 수요가 꾸준합니다. 위탁 주시면 검수와 오버홀을 거쳐 상태 그대로 정직하게 소개해 드리겠습니다.</t>
+  </si>
+  <si>
+    <t>드라켄은 크게 튀는 스펙은 아니지만 그만큼 실속 있다는 인식이 있어 수요가 꾸준합니다. 검수 후 상태를 투명하게 공개해서 내보내면, 구매하시는 분들도 믿고 결정하시더라고요.</t>
+  </si>
+  <si>
+    <t>아키스는 크게 튀는 스펙은 아니지만 그만큼 실속 있다는 인식이 있어 수요가 꾸준합니다. 위탁 주시면 검수와 오버홀을 거쳐 상태 그대로 정직하게 소개해 드리겠습니다.</t>
+  </si>
+  <si>
+    <t>코비를 처음 시작하는 분들이 많이 선택하다 보니, 중고 물량도 꾸준히 순환됩니다. 맡겨주시면 상태 점검부터 오버홀까지 해서, 제값 받고 팔릴 수 있게 도와드리겠습니다.</t>
+  </si>
+  <si>
+    <t>볼틱스 문어를 처음 시작하는 분들이 많이 선택하다 보니, 중고 물량도 꾸준히 순환됩니다. 특히 문어 하시는 분들 사이에서 선호도가 높습니다. 릴케어팜을 통해 위탁하시면 전문 검수와 정비를 거쳐 훨씬 수월하게 판매하실 수 있습니다.</t>
+  </si>
+  <si>
+    <t>레이오스를 처음 시작하는 분들이 많이 선택하다 보니, 중고 물량도 꾸준히 순환됩니다. 장르를 가리지 않고 두루 쓰인다는 점도 강점입니다. 위탁 주시면 검수와 오버홀을 거쳐 상태 그대로 정직하게 소개해 드리겠습니다.</t>
+  </si>
+  <si>
+    <t>제논 베이트는 소장 가치가 높은 상위 라인이라, 상태 좋은 개체는 오래 묵히지 않고 팔려나가는 편입니다. 특정 장르에 국한되지 않고 여러 상황에서 무난히 쓸 수 있습니다. 위탁 주시면 검수와 오버홀을 거쳐 상태 그대로 정직하게 소개해 드리겠습니다.</t>
+  </si>
+  <si>
+    <t>레보 SLC는 가격과 성능의 밸런스가 좋아서 꾸준히 찾는 분들이 있는 스테디셀러입니다. 릴케어팜에서 꼼꼼히 검수하고 손봐서 내보내면 구매자분들도 더 안심하고 선택하십니다.</t>
+  </si>
+  <si>
+    <t>레보 5X/5SX는 크게 튀는 스펙은 아니지만 그만큼 실속 있다는 인식이 있어 수요가 꾸준합니다. 배스 위주로 쓰시는 분들이 많이 찾는 편입니다. 저희 쪽에서 오버홀까지 마치고 판매하면 신뢰도가 올라가서 거래가 한결 수월해집니다.</t>
+  </si>
+  <si>
+    <t>솔티스테이지 Revo는 크게 튀는 스펙은 아니지만 그만큼 실속 있다는 인식이 있어 수요가 꾸준합니다. 선상 지깅 즐기는 분들에게 특히 반응이 좋은 편입니다. 위탁 주시면 검수와 오버홀을 거쳐 상태 그대로 정직하게 소개해 드리겠습니다.</t>
+  </si>
+  <si>
+    <t>레보 인쇼어를 두루 무난하게 쓸 수 있다는 평이 많아, 중고 거래도 활발한 편에 속합니다. 특정 장르에 국한되지 않고 여러 상황에서 무난히 쓸 수 있습니다. 위탁 주시면 검수와 오버홀을 거쳐 상태 그대로 정직하게 소개해 드리겠습니다.</t>
+  </si>
+  <si>
+    <t>록사니 BF8는 부담 없는 가격대라 입문자들이 많이 찾는 만큼, 중고로도 회전이 빠른 편입니다. 장르를 가리지 않고 두루 쓰인다는 점도 강점입니다. 맡겨주시면 상태 점검부터 오버홀까지 해서, 제값 받고 팔릴 수 있게 도와드리겠습니다.</t>
+  </si>
+  <si>
+    <t>프로맥스 4를 한 번 써본 분들의 만족도가 높다 보니, 재판매 수요도 꾸준한 편입니다. 특정 장르에 국한되지 않고 여러 상황에서 무난히 쓸 수 있습니다. 검수 후 상태를 투명하게 공개해서 내보내면, 구매하시는 분들도 믿고 결정하시더라고요.</t>
+  </si>
+  <si>
+    <t>블랙맥스 4는 부담 없는 가격대라 입문자들이 많이 찾는 만큼, 중고로도 회전이 빠른 편입니다. 장르를 가리지 않고 두루 쓰인다는 점도 강점입니다. 저희 쪽에서 오버홀까지 마치고 판매하면 신뢰도가 올라가서 거래가 한결 수월해집니다.</t>
+  </si>
+  <si>
+    <t>블루맥스/레드맥스는 가성비 좋은 입문작으로 알려져 있어서, 상태 좋은 매물은 크게 오래 기다리지 않고 나갑니다. 주꾸미·갑오징어 선상 즐기는 분들에게 특히 반응이 좋은 편입니다. 검수 후 상태를 투명하게 공개해서 내보내면, 구매하시는 분들도 믿고 결정하시더라고요.</t>
+  </si>
+  <si>
+    <t>꼬모도 SS를 두루 무난하게 쓸 수 있다는 평이 많아, 중고 거래도 활발한 편에 속합니다. 릴케어팜에서 꼼꼼히 검수하고 손봐서 내보내면 구매자분들도 더 안심하고 선택하십니다.</t>
+  </si>
+  <si>
+    <t>엘란 SW LIGHT는 가격과 성능의 밸런스가 좋아서 꾸준히 찾는 분들이 있는 스테디셀러입니다. 특정 장르에 국한되지 않고 여러 상황에서 무난히 쓸 수 있습니다. 저희 쪽에서 오버홀까지 마치고 판매하면 신뢰도가 올라가서 거래가 한결 수월해집니다.</t>
   </si>
 </sst>
 </file>
@@ -4599,7 +4900,7 @@
         <v>182</v>
       </c>
       <c r="I1" s="53" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="40.5" thickBot="1">
@@ -4627,6 +4928,9 @@
       <c r="H2" s="35" t="s">
         <v>186</v>
       </c>
+      <c r="I2" t="s">
+        <v>595</v>
+      </c>
     </row>
     <row r="3" spans="1:9" ht="40.5" thickBot="1">
       <c r="A3" s="15" t="s">
@@ -4653,6 +4957,9 @@
       <c r="H3" s="35" t="s">
         <v>188</v>
       </c>
+      <c r="I3" t="s">
+        <v>595</v>
+      </c>
     </row>
     <row r="4" spans="1:9" ht="27.75" thickBot="1">
       <c r="A4" s="15" t="s">
@@ -4679,6 +4986,9 @@
       <c r="H4" s="35" t="s">
         <v>191</v>
       </c>
+      <c r="I4" t="s">
+        <v>596</v>
+      </c>
     </row>
     <row r="5" spans="1:9" ht="27.75" thickBot="1">
       <c r="A5" s="15" t="s">
@@ -4705,6 +5015,9 @@
       <c r="H5" s="35" t="s">
         <v>194</v>
       </c>
+      <c r="I5" t="s">
+        <v>597</v>
+      </c>
     </row>
     <row r="6" spans="1:9" ht="27.75" thickBot="1">
       <c r="A6" s="15" t="s">
@@ -4731,6 +5044,9 @@
       <c r="H6" s="35" t="s">
         <v>197</v>
       </c>
+      <c r="I6" t="s">
+        <v>598</v>
+      </c>
     </row>
     <row r="7" spans="1:9" ht="17.25" thickBot="1">
       <c r="A7" s="15" t="s">
@@ -4757,6 +5073,9 @@
       <c r="H7" s="35" t="s">
         <v>199</v>
       </c>
+      <c r="I7" t="s">
+        <v>599</v>
+      </c>
     </row>
     <row r="8" spans="1:9" ht="27.75" thickBot="1">
       <c r="A8" s="15" t="s">
@@ -4783,6 +5102,9 @@
       <c r="H8" s="35" t="s">
         <v>202</v>
       </c>
+      <c r="I8" t="s">
+        <v>600</v>
+      </c>
     </row>
     <row r="9" spans="1:9" ht="27.75" thickBot="1">
       <c r="A9" s="15" t="s">
@@ -4809,6 +5131,9 @@
       <c r="H9" s="35" t="s">
         <v>204</v>
       </c>
+      <c r="I9" t="s">
+        <v>601</v>
+      </c>
     </row>
     <row r="10" spans="1:9" ht="27.75" thickBot="1">
       <c r="A10" s="15" t="s">
@@ -4835,6 +5160,9 @@
       <c r="H10" s="35" t="s">
         <v>207</v>
       </c>
+      <c r="I10" t="s">
+        <v>602</v>
+      </c>
     </row>
     <row r="11" spans="1:9" ht="27.75" thickBot="1">
       <c r="A11" s="15" t="s">
@@ -4861,6 +5189,9 @@
       <c r="H11" s="35" t="s">
         <v>210</v>
       </c>
+      <c r="I11" t="s">
+        <v>603</v>
+      </c>
     </row>
     <row r="12" spans="1:9" ht="17.25" thickBot="1">
       <c r="A12" s="15" t="s">
@@ -4887,6 +5218,9 @@
       <c r="H12" s="35" t="s">
         <v>212</v>
       </c>
+      <c r="I12" t="s">
+        <v>604</v>
+      </c>
     </row>
     <row r="13" spans="1:9" ht="27.75" thickBot="1">
       <c r="A13" s="15" t="s">
@@ -4913,6 +5247,9 @@
       <c r="H13" s="35" t="s">
         <v>214</v>
       </c>
+      <c r="I13" t="s">
+        <v>605</v>
+      </c>
     </row>
     <row r="14" spans="1:9" ht="17.25" thickBot="1">
       <c r="A14" s="15" t="s">
@@ -4939,6 +5276,9 @@
       <c r="H14" s="35" t="s">
         <v>216</v>
       </c>
+      <c r="I14" t="s">
+        <v>606</v>
+      </c>
     </row>
     <row r="15" spans="1:9" ht="17.25" thickBot="1">
       <c r="A15" s="15" t="s">
@@ -4965,6 +5305,9 @@
       <c r="H15" s="35" t="s">
         <v>219</v>
       </c>
+      <c r="I15" t="s">
+        <v>607</v>
+      </c>
     </row>
     <row r="16" spans="1:9" ht="27.75" thickBot="1">
       <c r="A16" s="15" t="s">
@@ -4991,8 +5334,11 @@
       <c r="H16" s="35" t="s">
         <v>222</v>
       </c>
-    </row>
-    <row r="17" spans="1:8" ht="27.75" thickBot="1">
+      <c r="I16" t="s">
+        <v>608</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" ht="27.75" thickBot="1">
       <c r="A17" s="15" t="s">
         <v>183</v>
       </c>
@@ -5017,8 +5363,11 @@
       <c r="H17" s="35" t="s">
         <v>225</v>
       </c>
-    </row>
-    <row r="18" spans="1:8" ht="27.75" thickBot="1">
+      <c r="I17" t="s">
+        <v>609</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="27.75" thickBot="1">
       <c r="A18" s="15" t="s">
         <v>183</v>
       </c>
@@ -5043,8 +5392,11 @@
       <c r="H18" s="35" t="s">
         <v>228</v>
       </c>
-    </row>
-    <row r="19" spans="1:8" ht="27.75" thickBot="1">
+      <c r="I18" t="s">
+        <v>610</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" ht="27.75" thickBot="1">
       <c r="A19" s="15" t="s">
         <v>183</v>
       </c>
@@ -5069,8 +5421,11 @@
       <c r="H19" s="35" t="s">
         <v>230</v>
       </c>
-    </row>
-    <row r="20" spans="1:8" ht="17.25" thickBot="1">
+      <c r="I19" t="s">
+        <v>611</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" ht="17.25" thickBot="1">
       <c r="A20" s="15" t="s">
         <v>183</v>
       </c>
@@ -5095,8 +5450,11 @@
       <c r="H20" s="35" t="s">
         <v>233</v>
       </c>
-    </row>
-    <row r="21" spans="1:8" ht="17.25" thickBot="1">
+      <c r="I20" t="s">
+        <v>612</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" ht="17.25" thickBot="1">
       <c r="A21" s="15" t="s">
         <v>183</v>
       </c>
@@ -5121,8 +5479,11 @@
       <c r="H21" s="35" t="s">
         <v>235</v>
       </c>
-    </row>
-    <row r="22" spans="1:8" ht="17.25" thickBot="1">
+      <c r="I21" t="s">
+        <v>613</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" ht="17.25" thickBot="1">
       <c r="A22" s="15" t="s">
         <v>236</v>
       </c>
@@ -5147,8 +5508,11 @@
       <c r="H22" s="35" t="s">
         <v>239</v>
       </c>
-    </row>
-    <row r="23" spans="1:8" ht="17.25" thickBot="1">
+      <c r="I22" t="s">
+        <v>614</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" ht="17.25" thickBot="1">
       <c r="A23" s="15" t="s">
         <v>236</v>
       </c>
@@ -5173,8 +5537,11 @@
       <c r="H23" s="35" t="s">
         <v>241</v>
       </c>
-    </row>
-    <row r="24" spans="1:8" ht="17.25" thickBot="1">
+      <c r="I23" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" ht="17.25" thickBot="1">
       <c r="A24" s="15" t="s">
         <v>236</v>
       </c>
@@ -5199,8 +5566,11 @@
       <c r="H24" s="35" t="s">
         <v>244</v>
       </c>
-    </row>
-    <row r="25" spans="1:8" ht="27.75" thickBot="1">
+      <c r="I24" t="s">
+        <v>616</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" ht="27.75" thickBot="1">
       <c r="A25" s="15" t="s">
         <v>236</v>
       </c>
@@ -5225,8 +5595,11 @@
       <c r="H25" s="35" t="s">
         <v>247</v>
       </c>
-    </row>
-    <row r="26" spans="1:8" ht="17.25" thickBot="1">
+      <c r="I25" t="s">
+        <v>617</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" ht="17.25" thickBot="1">
       <c r="A26" s="15" t="s">
         <v>236</v>
       </c>
@@ -5251,8 +5624,11 @@
       <c r="H26" s="35" t="s">
         <v>250</v>
       </c>
-    </row>
-    <row r="27" spans="1:8" ht="17.25" thickBot="1">
+      <c r="I26" t="s">
+        <v>618</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" ht="17.25" thickBot="1">
       <c r="A27" s="15" t="s">
         <v>236</v>
       </c>
@@ -5277,8 +5653,11 @@
       <c r="H27" s="35" t="s">
         <v>251</v>
       </c>
-    </row>
-    <row r="28" spans="1:8" ht="17.25" thickBot="1">
+      <c r="I27" t="s">
+        <v>618</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" ht="17.25" thickBot="1">
       <c r="A28" s="15" t="s">
         <v>236</v>
       </c>
@@ -5303,8 +5682,11 @@
       <c r="H28" s="35" t="s">
         <v>252</v>
       </c>
-    </row>
-    <row r="29" spans="1:8" ht="27.75" thickBot="1">
+      <c r="I28" t="s">
+        <v>618</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" ht="27.75" thickBot="1">
       <c r="A29" s="15" t="s">
         <v>236</v>
       </c>
@@ -5329,8 +5711,11 @@
       <c r="H29" s="35" t="s">
         <v>255</v>
       </c>
-    </row>
-    <row r="30" spans="1:8" ht="17.25" thickBot="1">
+      <c r="I29" t="s">
+        <v>619</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" ht="17.25" thickBot="1">
       <c r="A30" s="15" t="s">
         <v>236</v>
       </c>
@@ -5355,8 +5740,11 @@
       <c r="H30" s="35" t="s">
         <v>257</v>
       </c>
-    </row>
-    <row r="31" spans="1:8" ht="17.25" thickBot="1">
+      <c r="I30" t="s">
+        <v>620</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" ht="17.25" thickBot="1">
       <c r="A31" s="15" t="s">
         <v>236</v>
       </c>
@@ -5381,8 +5769,11 @@
       <c r="H31" s="35" t="s">
         <v>258</v>
       </c>
-    </row>
-    <row r="32" spans="1:8" ht="17.25" thickBot="1">
+      <c r="I31" t="s">
+        <v>621</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" ht="17.25" thickBot="1">
       <c r="A32" s="15" t="s">
         <v>236</v>
       </c>
@@ -5407,8 +5798,11 @@
       <c r="H32" s="35" t="s">
         <v>259</v>
       </c>
-    </row>
-    <row r="33" spans="1:8" ht="17.25" thickBot="1">
+      <c r="I32" t="s">
+        <v>622</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" ht="17.25" thickBot="1">
       <c r="A33" s="15" t="s">
         <v>236</v>
       </c>
@@ -5433,8 +5827,11 @@
       <c r="H33" s="35" t="s">
         <v>262</v>
       </c>
-    </row>
-    <row r="34" spans="1:8" ht="17.25" thickBot="1">
+      <c r="I33" t="s">
+        <v>623</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" ht="17.25" thickBot="1">
       <c r="A34" s="15" t="s">
         <v>236</v>
       </c>
@@ -5459,8 +5856,11 @@
       <c r="H34" s="36" t="s">
         <v>264</v>
       </c>
-    </row>
-    <row r="35" spans="1:8" ht="17.25" thickBot="1">
+      <c r="I34" t="s">
+        <v>624</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" ht="17.25" thickBot="1">
       <c r="A35" s="15" t="s">
         <v>236</v>
       </c>
@@ -5485,8 +5885,11 @@
       <c r="H35" s="35" t="s">
         <v>265</v>
       </c>
-    </row>
-    <row r="36" spans="1:8" ht="27.75" thickBot="1">
+      <c r="I35" t="s">
+        <v>624</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" ht="27.75" thickBot="1">
       <c r="A36" s="15" t="s">
         <v>236</v>
       </c>
@@ -5511,8 +5914,11 @@
       <c r="H36" s="35" t="s">
         <v>268</v>
       </c>
-    </row>
-    <row r="37" spans="1:8" ht="17.25" thickBot="1">
+      <c r="I36" t="s">
+        <v>625</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" ht="17.25" thickBot="1">
       <c r="A37" s="15" t="s">
         <v>236</v>
       </c>
@@ -5537,8 +5943,11 @@
       <c r="H37" s="35" t="s">
         <v>271</v>
       </c>
-    </row>
-    <row r="38" spans="1:8" ht="17.25" thickBot="1">
+      <c r="I37" t="s">
+        <v>626</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" ht="17.25" thickBot="1">
       <c r="A38" s="15" t="s">
         <v>236</v>
       </c>
@@ -5563,8 +5972,11 @@
       <c r="H38" s="35" t="s">
         <v>273</v>
       </c>
-    </row>
-    <row r="39" spans="1:8" ht="17.25" thickBot="1">
+      <c r="I38" t="s">
+        <v>627</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" ht="17.25" thickBot="1">
       <c r="A39" s="15" t="s">
         <v>236</v>
       </c>
@@ -5589,8 +6001,11 @@
       <c r="H39" s="35" t="s">
         <v>276</v>
       </c>
-    </row>
-    <row r="40" spans="1:8" ht="27.75" thickBot="1">
+      <c r="I39" t="s">
+        <v>628</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" ht="27.75" thickBot="1">
       <c r="A40" s="15" t="s">
         <v>236</v>
       </c>
@@ -5615,8 +6030,11 @@
       <c r="H40" s="35" t="s">
         <v>279</v>
       </c>
-    </row>
-    <row r="41" spans="1:8" ht="17.25" thickBot="1">
+      <c r="I40" t="s">
+        <v>629</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" ht="17.25" thickBot="1">
       <c r="A41" s="15" t="s">
         <v>280</v>
       </c>
@@ -5641,8 +6059,11 @@
       <c r="H41" s="35" t="s">
         <v>283</v>
       </c>
-    </row>
-    <row r="42" spans="1:8" ht="27.75" thickBot="1">
+      <c r="I41" t="s">
+        <v>630</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" ht="27.75" thickBot="1">
       <c r="A42" s="15" t="s">
         <v>280</v>
       </c>
@@ -5667,8 +6088,11 @@
       <c r="H42" s="35" t="s">
         <v>286</v>
       </c>
-    </row>
-    <row r="43" spans="1:8" ht="30.75" thickBot="1">
+      <c r="I42" t="s">
+        <v>631</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" ht="30.75" thickBot="1">
       <c r="A43" s="35" t="s">
         <v>280</v>
       </c>
@@ -5693,8 +6117,11 @@
       <c r="H43" s="36" t="s">
         <v>288</v>
       </c>
-    </row>
-    <row r="44" spans="1:8" ht="27.75" thickBot="1">
+      <c r="I43" t="s">
+        <v>632</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" ht="27.75" thickBot="1">
       <c r="A44" s="15" t="s">
         <v>280</v>
       </c>
@@ -5719,8 +6146,11 @@
       <c r="H44" s="35" t="s">
         <v>291</v>
       </c>
-    </row>
-    <row r="45" spans="1:8" ht="17.25" thickBot="1">
+      <c r="I44" t="s">
+        <v>633</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" ht="17.25" thickBot="1">
       <c r="A45" s="15" t="s">
         <v>280</v>
       </c>
@@ -5745,8 +6175,11 @@
       <c r="H45" s="35" t="s">
         <v>294</v>
       </c>
-    </row>
-    <row r="46" spans="1:8" ht="27.75" thickBot="1">
+      <c r="I45" t="s">
+        <v>634</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" ht="27.75" thickBot="1">
       <c r="A46" s="15" t="s">
         <v>280</v>
       </c>
@@ -5771,8 +6204,11 @@
       <c r="H46" s="35" t="s">
         <v>297</v>
       </c>
-    </row>
-    <row r="47" spans="1:8" ht="17.25" thickBot="1">
+      <c r="I46" t="s">
+        <v>635</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" ht="17.25" thickBot="1">
       <c r="A47" s="15" t="s">
         <v>280</v>
       </c>
@@ -5797,8 +6233,11 @@
       <c r="H47" s="35" t="s">
         <v>300</v>
       </c>
-    </row>
-    <row r="48" spans="1:8" ht="17.25" thickBot="1">
+      <c r="I47" t="s">
+        <v>636</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" ht="17.25" thickBot="1">
       <c r="A48" s="15" t="s">
         <v>280</v>
       </c>
@@ -5823,8 +6262,11 @@
       <c r="H48" s="35" t="s">
         <v>303</v>
       </c>
-    </row>
-    <row r="49" spans="1:8" ht="27.75" thickBot="1">
+      <c r="I48" t="s">
+        <v>637</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" ht="27.75" thickBot="1">
       <c r="A49" s="15" t="s">
         <v>280</v>
       </c>
@@ -5849,8 +6291,11 @@
       <c r="H49" s="35" t="s">
         <v>306</v>
       </c>
-    </row>
-    <row r="50" spans="1:8" ht="17.25" thickBot="1">
+      <c r="I49" t="s">
+        <v>638</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" ht="17.25" thickBot="1">
       <c r="A50" s="15" t="s">
         <v>280</v>
       </c>
@@ -5875,8 +6320,11 @@
       <c r="H50" s="35" t="s">
         <v>309</v>
       </c>
-    </row>
-    <row r="51" spans="1:8" ht="27.75" thickBot="1">
+      <c r="I50" t="s">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" ht="27.75" thickBot="1">
       <c r="A51" s="15" t="s">
         <v>97</v>
       </c>
@@ -5901,8 +6349,11 @@
       <c r="H51" s="35" t="s">
         <v>312</v>
       </c>
-    </row>
-    <row r="52" spans="1:8" ht="27.75" thickBot="1">
+      <c r="I51" t="s">
+        <v>640</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9" ht="27.75" thickBot="1">
       <c r="A52" s="15" t="s">
         <v>97</v>
       </c>
@@ -5927,8 +6378,11 @@
       <c r="H52" s="35" t="s">
         <v>315</v>
       </c>
-    </row>
-    <row r="53" spans="1:8" ht="17.25" thickBot="1">
+      <c r="I52" t="s">
+        <v>641</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9" ht="17.25" thickBot="1">
       <c r="A53" s="15" t="s">
         <v>97</v>
       </c>
@@ -5953,8 +6407,11 @@
       <c r="H53" s="35" t="s">
         <v>318</v>
       </c>
-    </row>
-    <row r="54" spans="1:8" ht="27.75" thickBot="1">
+      <c r="I53" t="s">
+        <v>642</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" ht="27.75" thickBot="1">
       <c r="A54" s="15" t="s">
         <v>97</v>
       </c>
@@ -5979,8 +6436,11 @@
       <c r="H54" s="35" t="s">
         <v>321</v>
       </c>
-    </row>
-    <row r="55" spans="1:8" ht="17.25" thickBot="1">
+      <c r="I54" t="s">
+        <v>643</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" ht="17.25" thickBot="1">
       <c r="A55" s="15" t="s">
         <v>97</v>
       </c>
@@ -6005,8 +6465,11 @@
       <c r="H55" s="35" t="s">
         <v>324</v>
       </c>
-    </row>
-    <row r="56" spans="1:8" ht="17.25" thickBot="1">
+      <c r="I55" t="s">
+        <v>644</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" ht="17.25" thickBot="1">
       <c r="A56" s="15" t="s">
         <v>97</v>
       </c>
@@ -6031,8 +6494,11 @@
       <c r="H56" s="35" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="57" spans="1:8" ht="17.25" thickBot="1">
+      <c r="I56" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" ht="17.25" thickBot="1">
       <c r="A57" s="15" t="s">
         <v>97</v>
       </c>
@@ -6057,8 +6523,11 @@
       <c r="H57" s="35" t="s">
         <v>329</v>
       </c>
-    </row>
-    <row r="58" spans="1:8" ht="27.75" thickBot="1">
+      <c r="I57" t="s">
+        <v>646</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" ht="27.75" thickBot="1">
       <c r="A58" s="15" t="s">
         <v>97</v>
       </c>
@@ -6083,8 +6552,11 @@
       <c r="H58" s="35" t="s">
         <v>332</v>
       </c>
-    </row>
-    <row r="59" spans="1:8" ht="27.75" thickBot="1">
+      <c r="I58" t="s">
+        <v>647</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" ht="27.75" thickBot="1">
       <c r="A59" s="15" t="s">
         <v>97</v>
       </c>
@@ -6109,8 +6581,11 @@
       <c r="H59" s="35" t="s">
         <v>335</v>
       </c>
-    </row>
-    <row r="60" spans="1:8" ht="17.25" thickBot="1">
+      <c r="I59" t="s">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" ht="17.25" thickBot="1">
       <c r="A60" s="15" t="s">
         <v>97</v>
       </c>
@@ -6135,8 +6610,11 @@
       <c r="H60" s="35" t="s">
         <v>338</v>
       </c>
-    </row>
-    <row r="61" spans="1:8" ht="27.75" thickBot="1">
+      <c r="I60" t="s">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9" ht="27.75" thickBot="1">
       <c r="A61" s="15" t="s">
         <v>339</v>
       </c>
@@ -6161,8 +6639,11 @@
       <c r="H61" s="35" t="s">
         <v>342</v>
       </c>
-    </row>
-    <row r="62" spans="1:8" ht="27.75" thickBot="1">
+      <c r="I61" t="s">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="62" spans="1:9" ht="27.75" thickBot="1">
       <c r="A62" s="15" t="s">
         <v>339</v>
       </c>
@@ -6187,8 +6668,11 @@
       <c r="H62" s="35" t="s">
         <v>345</v>
       </c>
-    </row>
-    <row r="63" spans="1:8" ht="27.75" thickBot="1">
+      <c r="I62" t="s">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="63" spans="1:9" ht="27.75" thickBot="1">
       <c r="A63" s="15" t="s">
         <v>339</v>
       </c>
@@ -6213,8 +6697,11 @@
       <c r="H63" s="35" t="s">
         <v>348</v>
       </c>
-    </row>
-    <row r="64" spans="1:8" ht="27.75" thickBot="1">
+      <c r="I63" t="s">
+        <v>652</v>
+      </c>
+    </row>
+    <row r="64" spans="1:9" ht="27.75" thickBot="1">
       <c r="A64" s="15" t="s">
         <v>339</v>
       </c>
@@ -6239,8 +6726,11 @@
       <c r="H64" s="35" t="s">
         <v>351</v>
       </c>
-    </row>
-    <row r="65" spans="1:8" ht="27.75" thickBot="1">
+      <c r="I64" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="65" spans="1:9" ht="27.75" thickBot="1">
       <c r="A65" s="15" t="s">
         <v>339</v>
       </c>
@@ -6265,8 +6755,11 @@
       <c r="H65" s="35" t="s">
         <v>354</v>
       </c>
-    </row>
-    <row r="66" spans="1:8" ht="40.5" thickBot="1">
+      <c r="I65" t="s">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="66" spans="1:9" ht="40.5" thickBot="1">
       <c r="A66" s="15" t="s">
         <v>339</v>
       </c>
@@ -6291,8 +6784,11 @@
       <c r="H66" s="35" t="s">
         <v>357</v>
       </c>
-    </row>
-    <row r="67" spans="1:8" ht="27.75" thickBot="1">
+      <c r="I66" t="s">
+        <v>655</v>
+      </c>
+    </row>
+    <row r="67" spans="1:9" ht="27.75" thickBot="1">
       <c r="A67" s="15" t="s">
         <v>339</v>
       </c>
@@ -6317,8 +6813,11 @@
       <c r="H67" s="35" t="s">
         <v>360</v>
       </c>
-    </row>
-    <row r="68" spans="1:8" ht="27.75" thickBot="1">
+      <c r="I67" t="s">
+        <v>656</v>
+      </c>
+    </row>
+    <row r="68" spans="1:9" ht="27.75" thickBot="1">
       <c r="A68" s="15" t="s">
         <v>339</v>
       </c>
@@ -6343,8 +6842,11 @@
       <c r="H68" s="35" t="s">
         <v>363</v>
       </c>
-    </row>
-    <row r="69" spans="1:8" ht="27.75" thickBot="1">
+      <c r="I68" t="s">
+        <v>657</v>
+      </c>
+    </row>
+    <row r="69" spans="1:9" ht="27.75" thickBot="1">
       <c r="A69" s="15" t="s">
         <v>339</v>
       </c>
@@ -6369,8 +6871,11 @@
       <c r="H69" s="35" t="s">
         <v>366</v>
       </c>
-    </row>
-    <row r="70" spans="1:8" ht="27.75" thickBot="1">
+      <c r="I69" t="s">
+        <v>658</v>
+      </c>
+    </row>
+    <row r="70" spans="1:9" ht="27.75" thickBot="1">
       <c r="A70" s="15" t="s">
         <v>367</v>
       </c>
@@ -6395,8 +6900,11 @@
       <c r="H70" s="35" t="s">
         <v>370</v>
       </c>
-    </row>
-    <row r="71" spans="1:8" ht="27.75" thickBot="1">
+      <c r="I70" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="71" spans="1:9" ht="27.75" thickBot="1">
       <c r="A71" s="15" t="s">
         <v>371</v>
       </c>
@@ -6420,6 +6928,9 @@
       </c>
       <c r="H71" s="35" t="s">
         <v>374</v>
+      </c>
+      <c r="I71" t="s">
+        <v>660</v>
       </c>
     </row>
   </sheetData>
@@ -6491,6 +7002,9 @@
       <c r="H2" s="36" t="s">
         <v>377</v>
       </c>
+      <c r="I2" t="s">
+        <v>559</v>
+      </c>
     </row>
     <row r="3" spans="1:9" ht="27.75" thickBot="1">
       <c r="A3" s="15" t="s">
@@ -6517,6 +7031,9 @@
       <c r="H3" s="36" t="s">
         <v>379</v>
       </c>
+      <c r="I3" t="s">
+        <v>559</v>
+      </c>
     </row>
     <row r="4" spans="1:9" ht="27.75" thickBot="1">
       <c r="A4" s="15" t="s">
@@ -6543,6 +7060,9 @@
       <c r="H4" s="36" t="s">
         <v>381</v>
       </c>
+      <c r="I4" t="s">
+        <v>559</v>
+      </c>
     </row>
     <row r="5" spans="1:9" ht="27.75" thickBot="1">
       <c r="A5" s="15" t="s">
@@ -6569,6 +7089,9 @@
       <c r="H5" s="36" t="s">
         <v>384</v>
       </c>
+      <c r="I5" t="s">
+        <v>560</v>
+      </c>
     </row>
     <row r="6" spans="1:9" ht="27.75" thickBot="1">
       <c r="A6" s="15" t="s">
@@ -6595,6 +7118,9 @@
       <c r="H6" s="36" t="s">
         <v>386</v>
       </c>
+      <c r="I6" t="s">
+        <v>561</v>
+      </c>
     </row>
     <row r="7" spans="1:9" ht="27.75" thickBot="1">
       <c r="A7" s="15" t="s">
@@ -6621,6 +7147,9 @@
       <c r="H7" s="36" t="s">
         <v>389</v>
       </c>
+      <c r="I7" t="s">
+        <v>562</v>
+      </c>
     </row>
     <row r="8" spans="1:9" ht="27.75" thickBot="1">
       <c r="A8" s="15" t="s">
@@ -6647,6 +7176,9 @@
       <c r="H8" s="36" t="s">
         <v>390</v>
       </c>
+      <c r="I8" t="s">
+        <v>563</v>
+      </c>
     </row>
     <row r="9" spans="1:9" ht="27.75" thickBot="1">
       <c r="A9" s="15" t="s">
@@ -6673,6 +7205,9 @@
       <c r="H9" s="36" t="s">
         <v>393</v>
       </c>
+      <c r="I9" t="s">
+        <v>564</v>
+      </c>
     </row>
     <row r="10" spans="1:9" ht="27.75" thickBot="1">
       <c r="A10" s="15" t="s">
@@ -6699,6 +7234,9 @@
       <c r="H10" s="36" t="s">
         <v>394</v>
       </c>
+      <c r="I10" t="s">
+        <v>565</v>
+      </c>
     </row>
     <row r="11" spans="1:9" ht="27.75" thickBot="1">
       <c r="A11" s="15" t="s">
@@ -6725,6 +7263,9 @@
       <c r="H11" s="36" t="s">
         <v>397</v>
       </c>
+      <c r="I11" t="s">
+        <v>566</v>
+      </c>
     </row>
     <row r="12" spans="1:9" ht="27.75" thickBot="1">
       <c r="A12" s="15" t="s">
@@ -6751,6 +7292,9 @@
       <c r="H12" s="36" t="s">
         <v>400</v>
       </c>
+      <c r="I12" t="s">
+        <v>567</v>
+      </c>
     </row>
     <row r="13" spans="1:9" ht="27.75" thickBot="1">
       <c r="A13" s="15" t="s">
@@ -6777,6 +7321,9 @@
       <c r="H13" s="36" t="s">
         <v>403</v>
       </c>
+      <c r="I13" t="s">
+        <v>568</v>
+      </c>
     </row>
     <row r="14" spans="1:9" ht="27.75" thickBot="1">
       <c r="A14" s="15" t="s">
@@ -6803,6 +7350,9 @@
       <c r="H14" s="36" t="s">
         <v>406</v>
       </c>
+      <c r="I14" t="s">
+        <v>569</v>
+      </c>
     </row>
     <row r="15" spans="1:9" ht="27.75" thickBot="1">
       <c r="A15" s="15" t="s">
@@ -6829,6 +7379,9 @@
       <c r="H15" s="36" t="s">
         <v>409</v>
       </c>
+      <c r="I15" t="s">
+        <v>570</v>
+      </c>
     </row>
     <row r="16" spans="1:9" ht="27.75" thickBot="1">
       <c r="A16" s="15" t="s">
@@ -6855,8 +7408,11 @@
       <c r="H16" s="36" t="s">
         <v>412</v>
       </c>
-    </row>
-    <row r="17" spans="1:8" ht="27.75" thickBot="1">
+      <c r="I16" t="s">
+        <v>571</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" ht="27.75" thickBot="1">
       <c r="A17" s="15" t="s">
         <v>280</v>
       </c>
@@ -6881,8 +7437,11 @@
       <c r="H17" s="36" t="s">
         <v>415</v>
       </c>
-    </row>
-    <row r="18" spans="1:8" ht="27.75" thickBot="1">
+      <c r="I17" t="s">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="27.75" thickBot="1">
       <c r="A18" s="15" t="s">
         <v>280</v>
       </c>
@@ -6907,8 +7466,11 @@
       <c r="H18" s="36" t="s">
         <v>418</v>
       </c>
-    </row>
-    <row r="19" spans="1:8" ht="27.75" thickBot="1">
+      <c r="I18" t="s">
+        <v>573</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" ht="27.75" thickBot="1">
       <c r="A19" s="15" t="s">
         <v>280</v>
       </c>
@@ -6933,8 +7495,11 @@
       <c r="H19" s="36" t="s">
         <v>421</v>
       </c>
-    </row>
-    <row r="20" spans="1:8" ht="27.75" thickBot="1">
+      <c r="I19" t="s">
+        <v>574</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" ht="27.75" thickBot="1">
       <c r="A20" s="15" t="s">
         <v>280</v>
       </c>
@@ -6959,8 +7524,11 @@
       <c r="H20" s="36" t="s">
         <v>424</v>
       </c>
-    </row>
-    <row r="21" spans="1:8" ht="27.75" thickBot="1">
+      <c r="I20" t="s">
+        <v>575</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" ht="27.75" thickBot="1">
       <c r="A21" s="15" t="s">
         <v>280</v>
       </c>
@@ -6985,8 +7553,11 @@
       <c r="H21" s="36" t="s">
         <v>427</v>
       </c>
-    </row>
-    <row r="22" spans="1:8" ht="27.75" thickBot="1">
+      <c r="I21" t="s">
+        <v>576</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" ht="27.75" thickBot="1">
       <c r="A22" s="15" t="s">
         <v>280</v>
       </c>
@@ -7011,8 +7582,11 @@
       <c r="H22" s="36" t="s">
         <v>430</v>
       </c>
-    </row>
-    <row r="23" spans="1:8" ht="27.75" thickBot="1">
+      <c r="I22" t="s">
+        <v>577</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" ht="27.75" thickBot="1">
       <c r="A23" s="15" t="s">
         <v>280</v>
       </c>
@@ -7037,8 +7611,11 @@
       <c r="H23" s="36" t="s">
         <v>432</v>
       </c>
-    </row>
-    <row r="24" spans="1:8" ht="27.75" thickBot="1">
+      <c r="I23" t="s">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" ht="27.75" thickBot="1">
       <c r="A24" s="15" t="s">
         <v>280</v>
       </c>
@@ -7063,8 +7640,11 @@
       <c r="H24" s="36" t="s">
         <v>435</v>
       </c>
-    </row>
-    <row r="25" spans="1:8" ht="27.75" thickBot="1">
+      <c r="I24" t="s">
+        <v>579</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" ht="27.75" thickBot="1">
       <c r="A25" s="15" t="s">
         <v>97</v>
       </c>
@@ -7089,8 +7669,11 @@
       <c r="H25" s="36" t="s">
         <v>438</v>
       </c>
-    </row>
-    <row r="26" spans="1:8" ht="27.75" thickBot="1">
+      <c r="I25" t="s">
+        <v>580</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" ht="27.75" thickBot="1">
       <c r="A26" s="15" t="s">
         <v>97</v>
       </c>
@@ -7115,8 +7698,11 @@
       <c r="H26" s="36" t="s">
         <v>441</v>
       </c>
-    </row>
-    <row r="27" spans="1:8" ht="17.25" thickBot="1">
+      <c r="I26" t="s">
+        <v>581</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" ht="17.25" thickBot="1">
       <c r="A27" s="15" t="s">
         <v>97</v>
       </c>
@@ -7141,8 +7727,11 @@
       <c r="H27" s="36" t="s">
         <v>444</v>
       </c>
-    </row>
-    <row r="28" spans="1:8" ht="27.75" thickBot="1">
+      <c r="I27" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" ht="27.75" thickBot="1">
       <c r="A28" s="15" t="s">
         <v>97</v>
       </c>
@@ -7167,8 +7756,11 @@
       <c r="H28" s="36" t="s">
         <v>447</v>
       </c>
-    </row>
-    <row r="29" spans="1:8" ht="27.75" thickBot="1">
+      <c r="I28" t="s">
+        <v>583</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" ht="27.75" thickBot="1">
       <c r="A29" s="15" t="s">
         <v>97</v>
       </c>
@@ -7193,8 +7785,11 @@
       <c r="H29" s="36" t="s">
         <v>450</v>
       </c>
-    </row>
-    <row r="30" spans="1:8" ht="27.75" thickBot="1">
+      <c r="I29" t="s">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" ht="27.75" thickBot="1">
       <c r="A30" s="15" t="s">
         <v>97</v>
       </c>
@@ -7219,8 +7814,11 @@
       <c r="H30" s="36" t="s">
         <v>453</v>
       </c>
-    </row>
-    <row r="31" spans="1:8" ht="27.75" thickBot="1">
+      <c r="I30" t="s">
+        <v>585</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" ht="27.75" thickBot="1">
       <c r="A31" s="15" t="s">
         <v>97</v>
       </c>
@@ -7245,8 +7843,11 @@
       <c r="H31" s="36" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="32" spans="1:8" ht="27.75" thickBot="1">
+      <c r="I31" t="s">
+        <v>586</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" ht="27.75" thickBot="1">
       <c r="A32" s="15" t="s">
         <v>339</v>
       </c>
@@ -7271,8 +7872,11 @@
       <c r="H32" s="36" t="s">
         <v>458</v>
       </c>
-    </row>
-    <row r="33" spans="1:8" ht="27.75" thickBot="1">
+      <c r="I32" t="s">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" ht="27.75" thickBot="1">
       <c r="A33" s="15" t="s">
         <v>339</v>
       </c>
@@ -7297,8 +7901,11 @@
       <c r="H33" s="36" t="s">
         <v>461</v>
       </c>
-    </row>
-    <row r="34" spans="1:8" ht="27.75" thickBot="1">
+      <c r="I33" t="s">
+        <v>588</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" ht="27.75" thickBot="1">
       <c r="A34" s="15" t="s">
         <v>339</v>
       </c>
@@ -7323,8 +7930,11 @@
       <c r="H34" s="36" t="s">
         <v>464</v>
       </c>
-    </row>
-    <row r="35" spans="1:8" ht="27.75" thickBot="1">
+      <c r="I34" t="s">
+        <v>589</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" ht="27.75" thickBot="1">
       <c r="A35" s="15" t="s">
         <v>339</v>
       </c>
@@ -7349,8 +7959,11 @@
       <c r="H35" s="36" t="s">
         <v>467</v>
       </c>
-    </row>
-    <row r="36" spans="1:8" ht="27.75" thickBot="1">
+      <c r="I35" t="s">
+        <v>590</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" ht="27.75" thickBot="1">
       <c r="A36" s="15" t="s">
         <v>339</v>
       </c>
@@ -7375,8 +7988,11 @@
       <c r="H36" s="36" t="s">
         <v>470</v>
       </c>
-    </row>
-    <row r="37" spans="1:8" ht="27.75" thickBot="1">
+      <c r="I36" t="s">
+        <v>591</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" ht="27.75" thickBot="1">
       <c r="A37" s="15" t="s">
         <v>339</v>
       </c>
@@ -7401,8 +8017,11 @@
       <c r="H37" s="36" t="s">
         <v>473</v>
       </c>
-    </row>
-    <row r="38" spans="1:8" ht="27.75" thickBot="1">
+      <c r="I37" t="s">
+        <v>592</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" ht="27.75" thickBot="1">
       <c r="A38" s="15" t="s">
         <v>339</v>
       </c>
@@ -7427,8 +8046,11 @@
       <c r="H38" s="36" t="s">
         <v>476</v>
       </c>
-    </row>
-    <row r="39" spans="1:8" ht="27.75" thickBot="1">
+      <c r="I38" t="s">
+        <v>593</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" ht="27.75" thickBot="1">
       <c r="A39" s="15" t="s">
         <v>477</v>
       </c>
@@ -7452,6 +8074,9 @@
       </c>
       <c r="H39" s="36" t="s">
         <v>480</v>
+      </c>
+      <c r="I39" t="s">
+        <v>594</v>
       </c>
     </row>
   </sheetData>

</xml_diff>